<commit_message>
added 0R resistors to the short circuit connections of the dsub pins. recreated output files for Rev02b
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_PER_deskbench_terminal/Rev02b/BOM/BOM_JLC-UZ_PER_deskbench_terminal.xlsx
+++ b/Project Outputs for UZ_PER_deskbench_terminal/Rev02b/BOM/BOM_JLC-UZ_PER_deskbench_terminal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_deskbench_terminal\Project Outputs for UZ_PER_deskbench_terminal\Rev02b\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{05900748-C22E-42C7-940E-84F7608925E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C71FF279-C475-427D-81D0-163EFA4E05AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-4320" windowWidth="30936" windowHeight="16776" xr2:uid="{A5D68247-DB97-4E71-9F80-C628BAEC1645}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="7270" xr2:uid="{A43613CB-79A8-4089-8066-4F2B9C586128}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_PER_deskbench_termin" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="46">
   <si>
     <t>Quantity</t>
   </si>
@@ -141,6 +141,24 @@
   </si>
   <si>
     <t>Fixed Mounting Block, 6 Pins, 5.08mm Pitch, 26-16 AWG</t>
+  </si>
+  <si>
+    <t>0R</t>
+  </si>
+  <si>
+    <t>R1, R2</t>
+  </si>
+  <si>
+    <t>UZgen</t>
+  </si>
+  <si>
+    <t>Generic resistor</t>
+  </si>
+  <si>
+    <t>R_0603_TE</t>
+  </si>
+  <si>
+    <t>UZgen_R_0603_0R</t>
   </si>
   <si>
     <t>Serial #</t>
@@ -554,8 +572,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21D1BA89-2A36-430D-993F-F08C1D275169}">
-  <dimension ref="A1:K8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B208A76-84C0-4F97-8D93-FF6994E91B52}">
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" customWidth="1"/>
@@ -777,7 +795,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>34</v>
@@ -788,7 +806,9 @@
       <c r="D8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="1"/>
+      <c r="E8" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="F8" s="2" t="s">
         <v>37</v>
       </c>
@@ -801,6 +821,33 @@
         <v>39</v>
       </c>
       <c r="K8" s="1"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" s="1">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="1"/>
+      <c r="F9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K9" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>